<commit_message>
update dashboard from Soccer365
</commit_message>
<xml_diff>
--- a/인천 2026 기록.xlsx
+++ b/인천 2026 기록.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://familyinter-my.sharepoint.com/personal/hwlee_familyinter_onmicrosoft_com/Documents/바탕 화면/프로젝트300/대시보드/인천 대시보드/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1065" documentId="11_8673CE99959C043A6D95B170604D1DCFD5B90D48" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{965D7F8E-F92F-4A1C-AC21-9527C0239A3B}"/>
+  <xr:revisionPtr revIDLastSave="2150" documentId="11_8673CE99959C043A6D95B170604D1DCFD5B90D48" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23400A68-04B9-4BBE-A10F-2B4BC21D2A4D}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8830" yWindow="1450" windowWidth="9600" windowHeight="5450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 토탈" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6018" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6036" uniqueCount="397">
   <si>
     <t>리그</t>
   </si>
@@ -1291,11 +1291,17 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>K리그1 2026 리그순위   (2026-09-09 - 28R 종료)</t>
+    <t>인천</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>인천</t>
+    <t>Kim Yeon-Soo</t>
+  </si>
+  <si>
+    <t>Leandro</t>
+  </si>
+  <si>
+    <t>K리그1 2026 리그순위   (2026-09-12 - 29R 진행 중)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -4961,6 +4967,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="기록표" displayName="기록표" ref="A42:E57" totalsRowShown="0" headerRowDxfId="84" headerRowBorderDxfId="83" tableBorderDxfId="82" totalsRowBorderDxfId="81">
   <tableColumns count="5">
@@ -5326,7 +5336,7 @@
         <v>1</v>
       </c>
       <c r="BI1" s="478" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="BJ1" s="477"/>
       <c r="BK1" s="477"/>
@@ -5593,11 +5603,11 @@
       </c>
       <c r="Y3" s="332">
         <f t="shared" ref="Y3:Y43" si="0">Z3+AA3</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Z3" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X3)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AA3" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X3)</f>
@@ -5605,7 +5615,7 @@
       </c>
       <c r="AB3" s="333">
         <f t="shared" ref="AB3:AB43" si="1">COUNTIF($M$3:$P$40,$X3)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AC3" s="334">
         <f t="shared" ref="AC3:AC43" si="2">COUNTIF($Q$3:$T$40,$X3)</f>
@@ -5613,15 +5623,15 @@
       </c>
       <c r="AD3" s="335">
         <f t="shared" ref="AD3:AD43" si="3">AB3+AC3</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AE3" s="332">
         <f t="shared" ref="AE3:AE43" si="4">AF3+AG3</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AF3" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X3)+Z3</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AG3" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X3)+AA3</f>
@@ -5629,7 +5639,7 @@
       </c>
       <c r="AH3" s="333">
         <f t="shared" ref="AH3:AH43" si="5">COUNTIF($M$3:$P$41,$X3)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AI3" s="334">
         <f t="shared" ref="AI3:AI43" si="6">COUNTIF($Q$3:$T$41,$X3)</f>
@@ -5637,7 +5647,7 @@
       </c>
       <c r="AJ3" s="335">
         <f t="shared" ref="AJ3:AJ43" si="7">AH3+AI3</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AM3" s="2" t="s">
         <v>45</v>
@@ -5724,10 +5734,10 @@
         <v>341</v>
       </c>
       <c r="BK3" s="469">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="BL3" s="469">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="BM3" s="469">
         <v>5</v>
@@ -5736,17 +5746,17 @@
         <v>5</v>
       </c>
       <c r="BO3" s="469">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="BP3" s="469">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="BQ3" s="469">
         <f>BO3-BP3</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="BR3" s="469">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:77">
@@ -5856,7 +5866,7 @@
       </c>
       <c r="AN4" s="2">
         <f>SUM(AO4:AQ4)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AO4" s="243">
         <f t="shared" si="8"/>
@@ -5868,7 +5878,7 @@
       </c>
       <c r="AQ4" s="342">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR4" s="352">
         <f>AO4*3+AP4</f>
@@ -5876,31 +5886,31 @@
       </c>
       <c r="AS4" s="23">
         <f>IFERROR(AO4/AN4,0)</f>
-        <v>0.38461538461538464</v>
+        <v>0.35714285714285715</v>
       </c>
       <c r="AT4" s="2">
         <f>SUMIFS($G$3:$G$40,$A$3:$A$40,"K리그",$F$3:$F$40,$AM4)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AU4" s="2">
         <f>SUMIFS($H$3:$H$40,$A$3:$A$40,"K리그",$F$3:$F$40,$AM4)</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="AV4" s="2">
         <f>AT4-AU4</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW4" s="434">
         <f>IFERROR(AR4/AN4,0)</f>
-        <v>1.4615384615384615</v>
+        <v>1.3571428571428572</v>
       </c>
       <c r="AX4" s="434">
         <f>IFERROR(AT4/AN4,0)</f>
-        <v>1.3846153846153846</v>
+        <v>1.3571428571428572</v>
       </c>
       <c r="AY4" s="434">
         <f>IFERROR(AU4/AN4,0)</f>
-        <v>1.1538461538461537</v>
+        <v>1.2142857142857142</v>
       </c>
       <c r="BA4" s="464" t="s">
         <v>53</v>
@@ -5936,10 +5946,10 @@
         <v>360</v>
       </c>
       <c r="BK4" s="470">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="BL4" s="470">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="BM4" s="470">
         <v>5</v>
@@ -5948,17 +5958,17 @@
         <v>10</v>
       </c>
       <c r="BO4" s="470">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="BP4" s="470">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="BQ4" s="470">
         <f>BO4-BP4</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BR4" s="470">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:77">
@@ -6011,7 +6021,7 @@
       </c>
       <c r="Y5" s="332">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Z5" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X5)</f>
@@ -6019,7 +6029,7 @@
       </c>
       <c r="AA5" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X5)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AB5" s="333">
         <f t="shared" si="1"/>
@@ -6035,7 +6045,7 @@
       </c>
       <c r="AE5" s="332">
         <f t="shared" si="4"/>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AF5" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X5)+Z5</f>
@@ -6043,7 +6053,7 @@
       </c>
       <c r="AG5" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X5)+AA5</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AH5" s="333">
         <f t="shared" si="5"/>
@@ -6062,7 +6072,7 @@
       </c>
       <c r="AN5" s="337">
         <f>SUM(AN3:AN4)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AO5" s="337">
         <f>SUM(AO3:AO4)</f>
@@ -6074,7 +6084,7 @@
       </c>
       <c r="AQ5" s="337">
         <f>SUM(AQ3:AQ4)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AR5" s="337">
         <f>SUM(AR3:AR4)</f>
@@ -6082,31 +6092,31 @@
       </c>
       <c r="AS5" s="349">
         <f>IFERROR(AO5/AN5,0)</f>
-        <v>0.37037037037037035</v>
+        <v>0.35714285714285715</v>
       </c>
       <c r="AT5" s="337">
         <f>SUM(AT3:AT4)</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AU5" s="337">
         <f>SUM(AU3:AU4)</f>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AV5" s="337">
         <f>SUM(AV3:AV4)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW5" s="435">
         <f>IFERROR(AR5/AN5,0)</f>
-        <v>1.3703703703703705</v>
+        <v>1.3214285714285714</v>
       </c>
       <c r="AX5" s="435">
         <f>IFERROR(AT5/AN5,0)</f>
-        <v>1.2592592592592593</v>
+        <v>1.25</v>
       </c>
       <c r="AY5" s="435">
         <f>IFERROR(AU5/AN5,0)</f>
-        <v>1.1111111111111112</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="BA5" s="464" t="s">
         <v>58</v>
@@ -6142,7 +6152,7 @@
         <v>365</v>
       </c>
       <c r="BK5" s="470">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="BL5" s="470">
         <v>11</v>
@@ -6151,17 +6161,17 @@
         <v>10</v>
       </c>
       <c r="BN5" s="470">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BO5" s="470">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="BP5" s="470">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="BQ5" s="470">
         <f>BO5-BP5</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="BR5" s="470">
         <v>43</v>
@@ -6221,7 +6231,7 @@
       </c>
       <c r="Y6" s="332">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Z6" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X6)</f>
@@ -6229,7 +6239,7 @@
       </c>
       <c r="AA6" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X6)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AB6" s="333">
         <f t="shared" si="1"/>
@@ -6245,7 +6255,7 @@
       </c>
       <c r="AE6" s="332">
         <f t="shared" si="4"/>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AF6" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X6)+Z6</f>
@@ -6253,7 +6263,7 @@
       </c>
       <c r="AG6" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X6)+AA6</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AH6" s="333">
         <f t="shared" si="5"/>
@@ -6302,7 +6312,7 @@
       </c>
       <c r="BB6" s="464">
         <f t="shared" si="9"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BC6" s="243">
         <f t="shared" si="10"/>
@@ -6314,7 +6324,7 @@
       </c>
       <c r="BE6" s="342">
         <f t="shared" si="10"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BF6" s="89">
         <f t="shared" si="11"/>
@@ -6322,7 +6332,7 @@
       </c>
       <c r="BG6" s="11">
         <f t="shared" si="12"/>
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="BI6" s="479">
         <v>4</v>
@@ -6331,29 +6341,29 @@
         <v>367</v>
       </c>
       <c r="BK6" s="479">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="BL6" s="479">
         <v>11</v>
       </c>
       <c r="BM6" s="479">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="BN6" s="479">
         <v>8</v>
       </c>
       <c r="BO6" s="479">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="BP6" s="479">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="BQ6" s="479">
         <f>BO6-BP6</f>
         <v>5</v>
       </c>
       <c r="BR6" s="479">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:77">
@@ -6406,11 +6416,11 @@
       </c>
       <c r="Y7" s="332">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z7" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X7)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AA7" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X7)</f>
@@ -6430,11 +6440,11 @@
       </c>
       <c r="AE7" s="332">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AF7" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X7)+Z7</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AG7" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X7)+AA7</f>
@@ -6609,11 +6619,11 @@
       </c>
       <c r="Y8" s="332">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z8" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X8)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AA8" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X8)</f>
@@ -6633,11 +6643,11 @@
       </c>
       <c r="AE8" s="332">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AF8" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X8)+Z8</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AG8" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X8)+AA8</f>
@@ -6731,29 +6741,29 @@
         <v>353</v>
       </c>
       <c r="BK8" s="479">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="BL8" s="479">
         <v>10</v>
       </c>
       <c r="BM8" s="479">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BN8" s="479">
         <v>10</v>
       </c>
       <c r="BO8" s="479">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="BP8" s="479">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="BQ8" s="479">
         <f>BO8-BP8</f>
         <v>9</v>
       </c>
       <c r="BR8" s="479">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:77">
@@ -6810,11 +6820,11 @@
       </c>
       <c r="Y9" s="332">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Z9" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X9)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AA9" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X9)</f>
@@ -6834,11 +6844,11 @@
       </c>
       <c r="AE9" s="332">
         <f t="shared" si="4"/>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AF9" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X9)+Z9</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AG9" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X9)+AA9</f>
@@ -6929,10 +6939,10 @@
         <v>7</v>
       </c>
       <c r="BJ9" s="471" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="BK9" s="471">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="BL9" s="471">
         <v>10</v>
@@ -6941,17 +6951,17 @@
         <v>7</v>
       </c>
       <c r="BN9" s="471">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BO9" s="471">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="BP9" s="471">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="BQ9" s="471">
         <f>BO9-BP9</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BR9" s="471">
         <v>37</v>
@@ -7133,29 +7143,29 @@
         <v>349</v>
       </c>
       <c r="BK10" s="479">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="BL10" s="479">
         <v>10</v>
       </c>
       <c r="BM10" s="479">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="BN10" s="479">
         <v>12</v>
       </c>
       <c r="BO10" s="479">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="BP10" s="479">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="BQ10" s="479">
         <f>BO10-BP10</f>
         <v>-7</v>
       </c>
       <c r="BR10" s="479">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:77">
@@ -7212,11 +7222,11 @@
       </c>
       <c r="Y11" s="332">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z11" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X11)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AA11" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X11)</f>
@@ -7236,11 +7246,11 @@
       </c>
       <c r="AE11" s="332">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AF11" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X11)+Z11</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AG11" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X11)+AA11</f>
@@ -7413,7 +7423,7 @@
       </c>
       <c r="Y12" s="332">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Z12" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X12)</f>
@@ -7421,7 +7431,7 @@
       </c>
       <c r="AA12" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X12)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AB12" s="333">
         <f t="shared" si="1"/>
@@ -7437,7 +7447,7 @@
       </c>
       <c r="AE12" s="332">
         <f t="shared" si="4"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AF12" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X12)+Z12</f>
@@ -7445,7 +7455,7 @@
       </c>
       <c r="AG12" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X12)+AA12</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AH12" s="333">
         <f t="shared" si="5"/>
@@ -7532,29 +7542,29 @@
         <v>362</v>
       </c>
       <c r="BK12" s="479">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="BL12" s="479">
         <v>7</v>
       </c>
       <c r="BM12" s="479">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BN12" s="479">
         <v>11</v>
       </c>
       <c r="BO12" s="479">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="BP12" s="479">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="BQ12" s="479">
         <f>BO12-BP12</f>
         <v>-7</v>
       </c>
       <c r="BR12" s="479">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:77">
@@ -7802,7 +7812,7 @@
       </c>
       <c r="Y14" s="332">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Z14" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X14)</f>
@@ -7810,7 +7820,7 @@
       </c>
       <c r="AA14" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X14)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AB14" s="333">
         <f t="shared" si="1"/>
@@ -7826,7 +7836,7 @@
       </c>
       <c r="AE14" s="332">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AF14" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X14)+Z14</f>
@@ -7834,7 +7844,7 @@
       </c>
       <c r="AG14" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X14)+AA14</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AH14" s="333">
         <f t="shared" si="5"/>
@@ -8059,7 +8069,7 @@
       </c>
       <c r="AN15" s="89">
         <f t="shared" si="13"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AO15" s="243">
         <f t="shared" si="14"/>
@@ -8071,7 +8081,7 @@
       </c>
       <c r="AQ15" s="351">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR15" s="352">
         <f t="shared" si="17"/>
@@ -8079,26 +8089,26 @@
       </c>
       <c r="AS15" s="23">
         <f>AO15/AN15</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="AT15" s="2">
         <f t="shared" si="18"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AU15" s="2">
         <f t="shared" si="19"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AV15" s="2">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="BA15" s="466" t="s">
         <v>60</v>
       </c>
       <c r="BB15" s="466">
         <f>SUM(BB3:BB14)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="BC15" s="243">
         <f>SUM(BC3:BC14)</f>
@@ -8110,7 +8120,7 @@
       </c>
       <c r="BE15" s="468">
         <f>SUM(BE3:BE14)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BF15" s="89">
         <f>SUM(BF3:BF14)</f>
@@ -8118,7 +8128,7 @@
       </c>
       <c r="BG15" s="11">
         <f t="shared" si="12"/>
-        <v>0.37037037037037035</v>
+        <v>0.35714285714285715</v>
       </c>
       <c r="BI15" s="476" t="s">
         <v>91</v>
@@ -8871,11 +8881,11 @@
       </c>
       <c r="Y22" s="332">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Z22" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X22)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AA22" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X22)</f>
@@ -8895,11 +8905,11 @@
       </c>
       <c r="AE22" s="332">
         <f t="shared" si="4"/>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AF22" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X22)+Z22</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AG22" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X22)+AA22</f>
@@ -8978,11 +8988,11 @@
       </c>
       <c r="Y23" s="332">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Z23" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X23)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AA23" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X23)</f>
@@ -9002,11 +9012,11 @@
       </c>
       <c r="AE23" s="332">
         <f t="shared" si="4"/>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AF23" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X23)+Z23</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AG23" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X23)+AA23</f>
@@ -9065,11 +9075,11 @@
       </c>
       <c r="Y24" s="332">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Z24" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X24)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AA24" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X24)</f>
@@ -9089,11 +9099,11 @@
       </c>
       <c r="AE24" s="332">
         <f t="shared" si="4"/>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AF24" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X24)+Z24</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AG24" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X24)+AA24</f>
@@ -9727,13 +9737,21 @@
       <c r="F31" s="267" t="s">
         <v>346</v>
       </c>
-      <c r="G31" s="266"/>
-      <c r="H31" s="266"/>
-      <c r="I31" s="380"/>
+      <c r="G31" s="266">
+        <v>1</v>
+      </c>
+      <c r="H31" s="266">
+        <v>2</v>
+      </c>
+      <c r="I31" s="380" t="s">
+        <v>33</v>
+      </c>
       <c r="J31" s="374"/>
       <c r="K31" s="266"/>
       <c r="L31" s="269"/>
-      <c r="M31" s="246"/>
+      <c r="M31" s="246" t="s">
+        <v>46</v>
+      </c>
       <c r="N31" s="270"/>
       <c r="O31" s="270"/>
       <c r="P31" s="271"/>
@@ -9742,7 +9760,9 @@
       <c r="S31" s="270"/>
       <c r="T31" s="270"/>
       <c r="U31" s="273"/>
-      <c r="V31" s="274"/>
+      <c r="V31" s="274" t="s">
+        <v>65</v>
+      </c>
       <c r="X31" s="329" t="s">
         <v>104</v>
       </c>
@@ -9922,11 +9942,11 @@
       </c>
       <c r="Y33" s="332">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Z33" s="132">
         <f>COUNTIF('출전기록 (26)'!C$2:M$39,'2026 토탈'!X33)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="AA33" s="132">
         <f>COUNTIF('출전기록 (26)'!N$2:S$39,'2026 토탈'!X33)</f>
@@ -9946,11 +9966,11 @@
       </c>
       <c r="AE33" s="332">
         <f t="shared" si="4"/>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AF33" s="132">
         <f>COUNTIF('출전기록 (26)'!W$2:AG$7,'2026 토탈'!X33)+Z33</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="AG33" s="132">
         <f>COUNTIF('출전기록 (26)'!AH$2:AM$7,'2026 토탈'!X33)+AA33</f>
@@ -36957,21 +36977,51 @@
       <c r="B30" s="264" t="s">
         <v>360</v>
       </c>
-      <c r="C30" s="297"/>
-      <c r="D30" s="243"/>
-      <c r="E30" s="243"/>
-      <c r="F30" s="243"/>
-      <c r="G30" s="243"/>
-      <c r="H30" s="243"/>
-      <c r="I30" s="243"/>
-      <c r="J30" s="243"/>
-      <c r="K30" s="243"/>
-      <c r="L30" s="243"/>
-      <c r="M30" s="298"/>
-      <c r="N30" s="110"/>
-      <c r="O30" s="2"/>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="159"/>
+      <c r="C30" s="297" t="s">
+        <v>106</v>
+      </c>
+      <c r="D30" s="243" t="s">
+        <v>89</v>
+      </c>
+      <c r="E30" s="243" t="s">
+        <v>394</v>
+      </c>
+      <c r="F30" s="243" t="s">
+        <v>64</v>
+      </c>
+      <c r="G30" s="243" t="s">
+        <v>52</v>
+      </c>
+      <c r="H30" s="243" t="s">
+        <v>74</v>
+      </c>
+      <c r="I30" s="243" t="s">
+        <v>71</v>
+      </c>
+      <c r="J30" s="243" t="s">
+        <v>51</v>
+      </c>
+      <c r="K30" s="243" t="s">
+        <v>395</v>
+      </c>
+      <c r="L30" s="243" t="s">
+        <v>46</v>
+      </c>
+      <c r="M30" s="298" t="s">
+        <v>81</v>
+      </c>
+      <c r="N30" s="110" t="s">
+        <v>59</v>
+      </c>
+      <c r="O30" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="P30" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q30" s="159" t="s">
+        <v>66</v>
+      </c>
       <c r="R30" s="159"/>
       <c r="S30" s="51"/>
       <c r="T30" s="1"/>

</xml_diff>